<commit_message>
Upload Download Summary - 2026-09-13 01:25:11
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 12, 2026</t>
+    <t>September 13, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18781838</v>
+        <v>18784476</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2755353</v>
+        <v>2758096</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1146928</v>
+        <v>1146967</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35243</v>
+        <v>35282</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202098</v>
+        <v>202201</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>48630</v>
+        <v>48733</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228372</v>
+        <v>228385</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>64877</v>
+        <v>64890</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>185776</v>
+        <v>185860</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>34971</v>
+        <v>35055</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196031</v>
+        <v>196049</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38655</v>
+        <v>38673</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>445961</v>
+        <v>446274</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>63213</v>
+        <v>63526</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>791397</v>
+        <v>791553</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>184029</v>
+        <v>184185</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95699</v>
+        <v>95810</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>6900</v>
+        <v>7011</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>253805</v>
+        <v>254411</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>68195</v>
+        <v>68801</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4063405</v>
+        <v>4064521</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1092813</v>
+        <v>1093929</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8006552</v>
+        <v>8007636</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>867209</v>
+        <v>868293</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3813118</v>
+        <v>3813668</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>644841</v>
+        <v>645391</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1329805</v>
+        <v>1329909</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>37930</v>
+        <v>38034</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>342555</v>
+        <v>342450</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1089331</v>
+        <v>1089204</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>86809</v>
+        <v>86682</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137072</v>
+        <v>137088</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>25751</v>
+        <v>25767</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6863066</v>
+        <v>6864089</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1219567</v>
+        <v>1220619</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17312485</v>
+        <v>17315091</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2721117</v>
+        <v>2723826</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-14 01:27:44
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 13, 2026</t>
+    <t>September 14, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18784476</v>
+        <v>18788214</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2758096</v>
+        <v>2761837</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1146967</v>
+        <v>1147038</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35282</v>
+        <v>35353</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202201</v>
+        <v>202315</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>48733</v>
+        <v>48847</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228385</v>
+        <v>228459</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>64890</v>
+        <v>64964</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>185860</v>
+        <v>185896</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35055</v>
+        <v>35091</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196049</v>
+        <v>196061</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38673</v>
+        <v>38685</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>446274</v>
+        <v>447192</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>63526</v>
+        <v>64444</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>791553</v>
+        <v>792840</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>184185</v>
+        <v>185472</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254411</v>
+        <v>254511</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>68801</v>
+        <v>68901</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4064521</v>
+        <v>4065151</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1093929</v>
+        <v>1094559</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8007636</v>
+        <v>8009280</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>868293</v>
+        <v>869937</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3813668</v>
+        <v>3814438</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>645391</v>
+        <v>646161</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1329909</v>
+        <v>1330182</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>38034</v>
+        <v>38307</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>342450</v>
+        <v>342447</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1089204</v>
+        <v>1089481</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>86682</v>
+        <v>86959</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137088</v>
+        <v>137235</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>25767</v>
+        <v>25914</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6864089</v>
+        <v>6865506</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1220619</v>
+        <v>1221973</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17315091</v>
+        <v>17318281</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2723826</v>
+        <v>2727057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-15 01:24:00
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 14, 2026</t>
+    <t>September 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18788214</v>
+        <v>18796902</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2761837</v>
+        <v>2770023</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147038</v>
+        <v>1147150</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35353</v>
+        <v>35465</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202315</v>
+        <v>202595</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>48847</v>
+        <v>49127</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228459</v>
+        <v>228598</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>64964</v>
+        <v>65103</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>185896</v>
+        <v>186003</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35091</v>
+        <v>35198</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196061</v>
+        <v>196083</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38685</v>
+        <v>38707</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>447192</v>
+        <v>447334</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>64444</v>
+        <v>64586</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>792840</v>
+        <v>792947</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>185472</v>
+        <v>185579</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95810</v>
+        <v>95868</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7011</v>
+        <v>7069</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254511</v>
+        <v>254556</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>68901</v>
+        <v>68946</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4065151</v>
+        <v>4067066</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1094559</v>
+        <v>1096474</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8009280</v>
+        <v>8011273</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>869937</v>
+        <v>871930</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3814438</v>
+        <v>3816943</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>646161</v>
+        <v>648666</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1330182</v>
+        <v>1331064</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>38307</v>
+        <v>39189</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>342447</v>
+        <v>342949</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1089481</v>
+        <v>1090322</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>86959</v>
+        <v>87800</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137235</v>
+        <v>137285</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>25914</v>
+        <v>25964</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6865506</v>
+        <v>6868653</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1221973</v>
+        <v>1225035</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17318281</v>
+        <v>17326582</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2727057</v>
+        <v>2734852</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-16 01:22:33
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 15, 2026</t>
+    <t>September 16, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18796902</v>
+        <v>18805957</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2770023</v>
+        <v>2778949</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147150</v>
+        <v>1147194</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35465</v>
+        <v>35509</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202595</v>
+        <v>202803</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49127</v>
+        <v>49335</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228598</v>
+        <v>228692</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65103</v>
+        <v>65197</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186003</v>
+        <v>186120</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35198</v>
+        <v>35315</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196083</v>
+        <v>196130</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38707</v>
+        <v>38754</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>447334</v>
+        <v>448056</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>64586</v>
+        <v>65308</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>792947</v>
+        <v>793072</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>185579</v>
+        <v>185704</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254556</v>
+        <v>254597</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>68946</v>
+        <v>68987</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4067066</v>
+        <v>4070661</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1096474</v>
+        <v>1100069</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8011273</v>
+        <v>8012474</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>871930</v>
+        <v>873131</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3816943</v>
+        <v>3819792</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>648666</v>
+        <v>651515</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1331064</v>
+        <v>1331446</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>39189</v>
+        <v>39571</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>342949</v>
+        <v>343078</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1090322</v>
+        <v>1091084</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>87800</v>
+        <v>88562</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137285</v>
+        <v>137422</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>25964</v>
+        <v>26101</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6868653</v>
+        <v>6872965</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1225035</v>
+        <v>1229494</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17326582</v>
+        <v>17335834</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2734852</v>
+        <v>2743823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-17 01:22:39
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 16, 2026</t>
+    <t>September 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18805957</v>
+        <v>18813674</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2778949</v>
+        <v>2786124</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147194</v>
+        <v>1147214</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35509</v>
+        <v>35529</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202803</v>
+        <v>202912</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49335</v>
+        <v>49444</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228692</v>
+        <v>228706</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65197</v>
+        <v>65211</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186120</v>
+        <v>186192</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35315</v>
+        <v>35387</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196130</v>
+        <v>196177</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38754</v>
+        <v>38801</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448056</v>
+        <v>448189</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65308</v>
+        <v>65441</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>793072</v>
+        <v>794351</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>185704</v>
+        <v>186983</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254597</v>
+        <v>254647</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>68987</v>
+        <v>69037</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4070661</v>
+        <v>4072625</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1100069</v>
+        <v>1102033</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8012474</v>
+        <v>8013774</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>873131</v>
+        <v>874431</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3819792</v>
+        <v>3821900</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>651515</v>
+        <v>653623</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1331446</v>
+        <v>1332277</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>39571</v>
+        <v>40402</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>343078</v>
+        <v>343620</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1091084</v>
+        <v>1092047</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>88562</v>
+        <v>89525</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137422</v>
+        <v>137431</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26101</v>
+        <v>26110</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6872965</v>
+        <v>6876029</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1229494</v>
+        <v>1232593</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17335834</v>
+        <v>17343461</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2743823</v>
+        <v>2750861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-18 01:22:56
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 17, 2026</t>
+    <t>September 18, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18813674</v>
+        <v>18820899</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2786124</v>
+        <v>2792678</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147214</v>
+        <v>1147664</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35529</v>
+        <v>35979</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202912</v>
+        <v>202960</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49444</v>
+        <v>49492</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228706</v>
+        <v>228720</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65211</v>
+        <v>65225</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186192</v>
+        <v>186343</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35387</v>
+        <v>35538</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196177</v>
+        <v>196189</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38801</v>
+        <v>38813</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448189</v>
+        <v>448326</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65441</v>
+        <v>65578</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794351</v>
+        <v>794460</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>186983</v>
+        <v>187092</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95868</v>
+        <v>95869</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7069</v>
+        <v>7070</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254647</v>
+        <v>254785</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>69037</v>
+        <v>69175</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4072625</v>
+        <v>4074291</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1102033</v>
+        <v>1103699</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8013774</v>
+        <v>8014867</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>874431</v>
+        <v>875524</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3821900</v>
+        <v>3824031</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>653623</v>
+        <v>655754</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1332277</v>
+        <v>1333240</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>40402</v>
+        <v>41365</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>343620</v>
+        <v>344291</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1092047</v>
+        <v>1092741</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>89525</v>
+        <v>90219</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137431</v>
+        <v>137438</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26110</v>
+        <v>26117</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6876029</v>
+        <v>6878646</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1232593</v>
+        <v>1235109</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17343461</v>
+        <v>17350394</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2750861</v>
+        <v>2757158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-19 01:19:49
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 18, 2026</t>
+    <t>September 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18820899</v>
+        <v>18828303</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2792678</v>
+        <v>2800011</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147664</v>
+        <v>1147686</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>35979</v>
+        <v>36001</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>202960</v>
+        <v>203043</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49492</v>
+        <v>49575</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228720</v>
+        <v>228815</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65225</v>
+        <v>65320</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186343</v>
+        <v>186380</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35538</v>
+        <v>35575</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196189</v>
+        <v>196227</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38813</v>
+        <v>38851</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448326</v>
+        <v>448349</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65578</v>
+        <v>65601</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794460</v>
+        <v>794572</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187092</v>
+        <v>187204</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95869</v>
+        <v>95873</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7070</v>
+        <v>7074</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254785</v>
+        <v>254836</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>69175</v>
+        <v>69226</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4074291</v>
+        <v>4076408</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1103699</v>
+        <v>1105816</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8014867</v>
+        <v>8016784</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>875524</v>
+        <v>877441</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3824031</v>
+        <v>3825957</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>655754</v>
+        <v>657680</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1333240</v>
+        <v>1333555</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>41365</v>
+        <v>41680</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344291</v>
+        <v>344362</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1092741</v>
+        <v>1093794</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>90219</v>
+        <v>91272</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137438</v>
+        <v>137443</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26117</v>
+        <v>26122</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6878646</v>
+        <v>6881776</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1235109</v>
+        <v>1238375</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17350394</v>
+        <v>17357987</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2757158</v>
+        <v>2764531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-20 01:26:08
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 19, 2026</t>
+    <t>September 20, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18828303</v>
+        <v>18832817</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2800011</v>
+        <v>2804480</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147686</v>
+        <v>1147746</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36001</v>
+        <v>36061</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203043</v>
+        <v>203135</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49575</v>
+        <v>49667</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228815</v>
+        <v>228822</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65320</v>
+        <v>65327</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186380</v>
+        <v>186398</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35575</v>
+        <v>35593</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196227</v>
+        <v>196244</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38851</v>
+        <v>38868</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448349</v>
+        <v>448400</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65601</v>
+        <v>65652</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794572</v>
+        <v>794680</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187204</v>
+        <v>187312</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254836</v>
+        <v>254848</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>69226</v>
+        <v>69238</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4076408</v>
+        <v>4077210</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1105816</v>
+        <v>1106618</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8016784</v>
+        <v>8018690</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>877441</v>
+        <v>879347</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3825957</v>
+        <v>3826951</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>657680</v>
+        <v>658674</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1333555</v>
+        <v>1334070</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>41680</v>
+        <v>42195</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344362</v>
+        <v>344407</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1093794</v>
+        <v>1094044</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>91272</v>
+        <v>91522</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137443</v>
+        <v>137445</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26122</v>
+        <v>26124</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6881776</v>
+        <v>6883173</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1238375</v>
+        <v>1239658</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17357987</v>
+        <v>17362149</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2764531</v>
+        <v>2768655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-21 01:25:54
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 20, 2026</t>
+    <t>September 21, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18832817</v>
+        <v>18836328</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2804480</v>
+        <v>2807956</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147746</v>
+        <v>1147796</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36061</v>
+        <v>36111</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203135</v>
+        <v>203205</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49667</v>
+        <v>49737</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228822</v>
+        <v>228842</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65327</v>
+        <v>65347</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186398</v>
+        <v>186454</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35593</v>
+        <v>35649</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196244</v>
+        <v>196254</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38868</v>
+        <v>38878</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448400</v>
+        <v>448450</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65652</v>
+        <v>65702</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794680</v>
+        <v>794797</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187312</v>
+        <v>187429</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>254848</v>
+        <v>255608</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>69238</v>
+        <v>69998</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4077210</v>
+        <v>4077906</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1106618</v>
+        <v>1107314</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8018690</v>
+        <v>8020070</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>879347</v>
+        <v>880727</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3826951</v>
+        <v>3827743</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>658674</v>
+        <v>659466</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1334070</v>
+        <v>1334415</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>42195</v>
+        <v>42540</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344407</v>
+        <v>344442</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1094044</v>
+        <v>1094213</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>91522</v>
+        <v>91691</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137445</v>
+        <v>137539</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26124</v>
+        <v>26218</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6883173</v>
+        <v>6884378</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1239658</v>
+        <v>1240790</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17362149</v>
+        <v>17365255</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2768655</v>
+        <v>2771791</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-22 01:21:16
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 21, 2026</t>
+    <t>September 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18836328</v>
+        <v>18843804</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2807956</v>
+        <v>2814977</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147796</v>
+        <v>1147834</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36111</v>
+        <v>36149</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203205</v>
+        <v>203472</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>49737</v>
+        <v>50004</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228842</v>
+        <v>228912</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65347</v>
+        <v>65417</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186454</v>
+        <v>186546</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35649</v>
+        <v>35741</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196254</v>
+        <v>196293</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38878</v>
+        <v>38917</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448450</v>
+        <v>448694</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65702</v>
+        <v>65946</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794797</v>
+        <v>794915</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187429</v>
+        <v>187547</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95873</v>
+        <v>95929</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7074</v>
+        <v>7130</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>255608</v>
+        <v>255717</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>69998</v>
+        <v>70107</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4077906</v>
+        <v>4080174</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1107314</v>
+        <v>1109582</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8020070</v>
+        <v>8021445</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>880727</v>
+        <v>882102</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3827743</v>
+        <v>3829577</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>659466</v>
+        <v>661300</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1334415</v>
+        <v>1335103</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>42540</v>
+        <v>43228</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344442</v>
+        <v>344897</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1094213</v>
+        <v>1094978</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>91691</v>
+        <v>92456</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137539</v>
+        <v>137630</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26218</v>
+        <v>26309</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6884378</v>
+        <v>6887831</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1240790</v>
+        <v>1244158</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17365255</v>
+        <v>17372222</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2771791</v>
+        <v>2778392</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-23 01:22:12
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 22, 2026</t>
+    <t>September 23, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18843804</v>
+        <v>18849695</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2814977</v>
+        <v>2820555</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147834</v>
+        <v>1147935</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36149</v>
+        <v>36250</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203472</v>
+        <v>203577</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50004</v>
+        <v>50109</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228912</v>
+        <v>228927</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65417</v>
+        <v>65432</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186546</v>
+        <v>186615</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35741</v>
+        <v>35810</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196293</v>
+        <v>196322</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38917</v>
+        <v>38946</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448694</v>
+        <v>448709</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65946</v>
+        <v>65961</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>794915</v>
+        <v>795022</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187547</v>
+        <v>187654</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95929</v>
+        <v>95932</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7130</v>
+        <v>7133</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>255717</v>
+        <v>255849</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>70107</v>
+        <v>70239</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4080174</v>
+        <v>4082424</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1109582</v>
+        <v>1111832</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8021445</v>
+        <v>8022366</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>882102</v>
+        <v>883023</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3829577</v>
+        <v>3831014</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>661300</v>
+        <v>662737</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1335103</v>
+        <v>1335577</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>43228</v>
+        <v>43702</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344897</v>
+        <v>345210</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1094978</v>
+        <v>1095470</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>92456</v>
+        <v>92948</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137630</v>
+        <v>137634</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26309</v>
+        <v>26313</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6887831</v>
+        <v>6890686</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1244158</v>
+        <v>1247010</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17372222</v>
+        <v>17377992</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2778392</v>
+        <v>2783857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-24 01:22:20
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 23, 2026</t>
+    <t>September 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18849695</v>
+        <v>18853139</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2820555</v>
+        <v>2824217</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1147935</v>
+        <v>1148011</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36250</v>
+        <v>36326</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203577</v>
+        <v>203695</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50109</v>
+        <v>50227</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228927</v>
+        <v>228955</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65432</v>
+        <v>65460</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186615</v>
+        <v>186673</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35810</v>
+        <v>35868</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196322</v>
+        <v>196355</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38946</v>
+        <v>38979</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448709</v>
+        <v>448750</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>65961</v>
+        <v>66002</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>795022</v>
+        <v>795143</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187654</v>
+        <v>187775</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95932</v>
+        <v>95933</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7133</v>
+        <v>7134</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>255849</v>
+        <v>256160</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>70239</v>
+        <v>70550</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4082424</v>
+        <v>4084615</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1111832</v>
+        <v>1114023</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8022366</v>
+        <v>8022744</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>883023</v>
+        <v>883401</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3831014</v>
+        <v>3832082</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>662737</v>
+        <v>663805</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1335577</v>
+        <v>1335512</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>43702</v>
+        <v>43637</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>345210</v>
+        <v>344992</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1095470</v>
+        <v>1095555</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>92948</v>
+        <v>93033</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137634</v>
+        <v>137639</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26313</v>
+        <v>26318</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6890686</v>
+        <v>6892392</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1247010</v>
+        <v>1248928</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17377992</v>
+        <v>17382216</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2783857</v>
+        <v>2788089</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-25 01:21:48
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 24, 2026</t>
+    <t>September 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18853139</v>
+        <v>18861480</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2824217</v>
+        <v>2832110</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148011</v>
+        <v>1148075</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36326</v>
+        <v>36390</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203695</v>
+        <v>203815</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50227</v>
+        <v>50347</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228955</v>
+        <v>228989</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65460</v>
+        <v>65494</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186673</v>
+        <v>186768</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35868</v>
+        <v>35963</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196355</v>
+        <v>196395</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>38979</v>
+        <v>39019</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448750</v>
+        <v>448882</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>66002</v>
+        <v>66134</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>795143</v>
+        <v>795271</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187775</v>
+        <v>187903</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95933</v>
+        <v>95936</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7134</v>
+        <v>7137</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256160</v>
+        <v>256266</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>70550</v>
+        <v>70656</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4084615</v>
+        <v>4086445</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1114023</v>
+        <v>1115853</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8022744</v>
+        <v>8024326</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>883401</v>
+        <v>884983</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3832082</v>
+        <v>3834680</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>663805</v>
+        <v>666403</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1335512</v>
+        <v>1336239</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>43637</v>
+        <v>44364</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>344992</v>
+        <v>345440</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1095555</v>
+        <v>1096690</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>93033</v>
+        <v>94168</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137639</v>
+        <v>137660</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26318</v>
+        <v>26339</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6892392</v>
+        <v>6895498</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1248928</v>
+        <v>1252009</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17382216</v>
+        <v>17390399</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2788089</v>
+        <v>2795841</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-26 01:21:02
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 25, 2026</t>
+    <t>September 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18861480</v>
+        <v>18872168</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2832110</v>
+        <v>2842019</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148075</v>
+        <v>1148134</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36390</v>
+        <v>36449</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203815</v>
+        <v>203868</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50347</v>
+        <v>50400</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>228989</v>
+        <v>229061</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65494</v>
+        <v>65566</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186768</v>
+        <v>186857</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>35963</v>
+        <v>36052</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196395</v>
+        <v>196445</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39019</v>
+        <v>39069</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>448882</v>
+        <v>449002</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>66134</v>
+        <v>66254</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>795271</v>
+        <v>795468</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>187903</v>
+        <v>188100</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95936</v>
+        <v>95937</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7137</v>
+        <v>7138</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256266</v>
+        <v>256750</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>70656</v>
+        <v>71140</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4086445</v>
+        <v>4088774</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1115853</v>
+        <v>1118182</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8024326</v>
+        <v>8026589</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>884983</v>
+        <v>887246</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3834680</v>
+        <v>3837377</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>666403</v>
+        <v>669100</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1336239</v>
+        <v>1337226</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>44364</v>
+        <v>45351</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>345440</v>
+        <v>346219</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1096690</v>
+        <v>1098307</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>94168</v>
+        <v>95785</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137660</v>
+        <v>137676</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26339</v>
+        <v>26355</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6895498</v>
+        <v>6899488</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1252009</v>
+        <v>1256004</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17390399</v>
+        <v>17401055</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2795841</v>
+        <v>2805706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-27 01:30:08
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 26, 2026</t>
+    <t>September 27, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18872168</v>
+        <v>18875222</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2842019</v>
+        <v>2845338</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148134</v>
+        <v>1148380</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36449</v>
+        <v>36695</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203868</v>
+        <v>203925</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50400</v>
+        <v>50457</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229061</v>
+        <v>229083</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65566</v>
+        <v>65588</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186857</v>
+        <v>186906</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36052</v>
+        <v>36101</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196445</v>
+        <v>196457</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39069</v>
+        <v>39081</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>449002</v>
+        <v>449224</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>66254</v>
+        <v>66476</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>795468</v>
+        <v>796064</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>188100</v>
+        <v>188696</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95937</v>
+        <v>95939</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7138</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256750</v>
+        <v>256847</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71140</v>
+        <v>71237</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4088774</v>
+        <v>4089977</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1118182</v>
+        <v>1119385</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8026589</v>
+        <v>8027382</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>887246</v>
+        <v>888039</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3837377</v>
+        <v>3837917</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>669100</v>
+        <v>669640</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1337226</v>
+        <v>1337258</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>45351</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346219</v>
+        <v>345954</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1098307</v>
+        <v>1098888</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>95785</v>
+        <v>96366</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137676</v>
+        <v>137846</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26355</v>
+        <v>26525</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6899488</v>
+        <v>6901599</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1256004</v>
+        <v>1258049</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17401055</v>
+        <v>17403721</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2805706</v>
+        <v>2808698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-28 01:31:53
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 27, 2026</t>
+    <t>September 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18875222</v>
+        <v>18878327</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2845338</v>
+        <v>2848649</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148380</v>
+        <v>1148400</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36695</v>
+        <v>36715</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203925</v>
+        <v>203963</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50457</v>
+        <v>50495</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229083</v>
+        <v>229091</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65588</v>
+        <v>65596</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186906</v>
+        <v>186953</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36101</v>
+        <v>36148</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196457</v>
+        <v>196490</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39081</v>
+        <v>39114</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>449224</v>
+        <v>450247</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>66476</v>
+        <v>67499</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>796064</v>
+        <v>796196</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>188696</v>
+        <v>188828</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95939</v>
+        <v>95940</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7140</v>
+        <v>7141</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256847</v>
+        <v>256884</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71237</v>
+        <v>71274</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4089977</v>
+        <v>4091198</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1119385</v>
+        <v>1120606</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8027382</v>
+        <v>8028629</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>888039</v>
+        <v>889286</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3837917</v>
+        <v>3838350</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>669640</v>
+        <v>670073</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1337258</v>
+        <v>1337361</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>45383</v>
+        <v>45486</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>345954</v>
+        <v>345748</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1098888</v>
+        <v>1099182</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>96366</v>
+        <v>96660</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137846</v>
+        <v>137859</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26525</v>
+        <v>26538</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6901599</v>
+        <v>6902962</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1258049</v>
+        <v>1259469</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17403721</v>
+        <v>17407055</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2808698</v>
+        <v>2812161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-29 01:27:34
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 28, 2026</t>
+    <t>September 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18878327</v>
+        <v>18890057</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2848649</v>
+        <v>2859481</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148400</v>
+        <v>1148438</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36715</v>
+        <v>36753</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>203963</v>
+        <v>204253</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50495</v>
+        <v>50785</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229091</v>
+        <v>229170</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65596</v>
+        <v>65675</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>186953</v>
+        <v>187083</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36148</v>
+        <v>36278</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196490</v>
+        <v>196517</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39114</v>
+        <v>39141</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>450247</v>
+        <v>450293</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>67499</v>
+        <v>67545</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>796196</v>
+        <v>796302</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>188828</v>
+        <v>188934</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256884</v>
+        <v>256967</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71274</v>
+        <v>71357</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4091198</v>
+        <v>4094465</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1120606</v>
+        <v>1123873</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8028629</v>
+        <v>8031466</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>889286</v>
+        <v>892123</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3838350</v>
+        <v>3840911</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>670073</v>
+        <v>672634</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1337361</v>
+        <v>1338579</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>45486</v>
+        <v>46704</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>345748</v>
+        <v>346646</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1099182</v>
+        <v>1100127</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>96660</v>
+        <v>97605</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137859</v>
+        <v>137863</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26538</v>
+        <v>26542</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6902962</v>
+        <v>6907009</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1259469</v>
+        <v>1263660</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17407055</v>
+        <v>17419091</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2812161</v>
+        <v>2823158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-09-30 01:30:58
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 29, 2026</t>
+    <t>September 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18890057</v>
+        <v>18895991</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2859481</v>
+        <v>2865472</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148438</v>
+        <v>1148707</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>36753</v>
+        <v>37022</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204253</v>
+        <v>204343</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50785</v>
+        <v>50875</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229170</v>
+        <v>229384</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65675</v>
+        <v>65889</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187083</v>
+        <v>187170</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36278</v>
+        <v>36365</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196517</v>
+        <v>196542</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39141</v>
+        <v>39166</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>450293</v>
+        <v>450361</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>67545</v>
+        <v>67613</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>796302</v>
+        <v>796771</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>188934</v>
+        <v>189403</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95940</v>
+        <v>95941</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7141</v>
+        <v>7142</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>256967</v>
+        <v>257065</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71357</v>
+        <v>71455</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4094465</v>
+        <v>4097333</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1123873</v>
+        <v>1126741</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8031466</v>
+        <v>8032771</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>892123</v>
+        <v>893428</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3840911</v>
+        <v>3842075</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>672634</v>
+        <v>673798</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1338579</v>
+        <v>1339004</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>46704</v>
+        <v>47129</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346646</v>
+        <v>346589</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1100127</v>
+        <v>1100340</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>97605</v>
+        <v>97818</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137863</v>
+        <v>137879</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26542</v>
+        <v>26558</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6907009</v>
+        <v>6910000</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1263660</v>
+        <v>1266671</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17419091</v>
+        <v>17425229</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2823158</v>
+        <v>2829239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-01 01:37:55
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 30, 2026</t>
+    <t>October 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18895991</v>
+        <v>18902793</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2865472</v>
+        <v>2872240</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148707</v>
+        <v>1148745</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37022</v>
+        <v>37060</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204343</v>
+        <v>204468</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>50875</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229384</v>
+        <v>229744</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>65889</v>
+        <v>66249</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187170</v>
+        <v>187243</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36365</v>
+        <v>36438</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196542</v>
+        <v>196583</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39166</v>
+        <v>39207</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>450361</v>
+        <v>450414</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>67613</v>
+        <v>67666</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>796771</v>
+        <v>798518</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>189403</v>
+        <v>191150</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95941</v>
+        <v>95945</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7142</v>
+        <v>7146</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>257065</v>
+        <v>257147</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71455</v>
+        <v>71537</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4097333</v>
+        <v>4100043</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1126741</v>
+        <v>1129451</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8032771</v>
+        <v>8034535</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>893428</v>
+        <v>895192</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3842075</v>
+        <v>3843632</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>673798</v>
+        <v>675355</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1339004</v>
+        <v>1339291</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>47129</v>
+        <v>47416</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346589</v>
+        <v>346623</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1100340</v>
+        <v>1100537</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>97818</v>
+        <v>98015</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>137879</v>
+        <v>138132</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26558</v>
+        <v>26811</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6910000</v>
+        <v>6912626</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1266671</v>
+        <v>1269405</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17425229</v>
+        <v>17432404</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2829239</v>
+        <v>2836288</v>
       </c>
     </row>
   </sheetData>
@@ -1177,7 +1177,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-02 01:28:03
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 1, 2026</t>
+    <t>October 2, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18902793</v>
+        <v>18909681</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2872240</v>
+        <v>2879409</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148745</v>
+        <v>1148966</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37060</v>
+        <v>37281</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204468</v>
+        <v>204589</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51000</v>
+        <v>51121</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>229744</v>
+        <v>230302</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>66249</v>
+        <v>66807</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187243</v>
+        <v>187289</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36438</v>
+        <v>36484</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196583</v>
+        <v>196604</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39207</v>
+        <v>39228</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>450414</v>
+        <v>450456</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>67666</v>
+        <v>67708</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>798518</v>
+        <v>798755</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>191150</v>
+        <v>191387</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>95945</v>
+        <v>96010</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7146</v>
+        <v>7211</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>257147</v>
+        <v>257222</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71537</v>
+        <v>71612</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4100043</v>
+        <v>4102996</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1129451</v>
+        <v>1132404</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8034535</v>
+        <v>8036455</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>895192</v>
+        <v>897112</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3843632</v>
+        <v>3844665</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>675355</v>
+        <v>676388</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1339291</v>
+        <v>1339392</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>47416</v>
+        <v>47517</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346623</v>
+        <v>346342</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1100537</v>
+        <v>1100883</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>98015</v>
+        <v>98361</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>138132</v>
+        <v>138948</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>26811</v>
+        <v>27627</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6912626</v>
+        <v>6915371</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1269405</v>
+        <v>1272423</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17432404</v>
+        <v>17440175</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2836288</v>
+        <v>2844011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-03 01:24:42
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 2, 2026</t>
+    <t>October 3, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18909681</v>
+        <v>18916133</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2879409</v>
+        <v>2885965</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1148966</v>
+        <v>1149057</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37281</v>
+        <v>37372</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204589</v>
+        <v>204712</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51121</v>
+        <v>51244</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>230302</v>
+        <v>230479</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>66807</v>
+        <v>66984</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187289</v>
+        <v>187396</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36484</v>
+        <v>36591</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196604</v>
+        <v>196680</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39228</v>
+        <v>39304</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>450456</v>
+        <v>451167</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>67708</v>
+        <v>68419</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>798755</v>
+        <v>800458</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>191387</v>
+        <v>193090</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96010</v>
+        <v>96069</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7211</v>
+        <v>7270</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>257222</v>
+        <v>257632</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>71612</v>
+        <v>72022</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4102996</v>
+        <v>4105463</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1132404</v>
+        <v>1134871</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8036455</v>
+        <v>8038316</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>897112</v>
+        <v>898973</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3844665</v>
+        <v>3845869</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>676388</v>
+        <v>677592</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1339392</v>
+        <v>1339666</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>47517</v>
+        <v>47791</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346342</v>
+        <v>346238</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1100883</v>
+        <v>1101391</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>98361</v>
+        <v>98869</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>138948</v>
+        <v>139190</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>27627</v>
+        <v>27869</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6915371</v>
+        <v>6918507</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1272423</v>
+        <v>1275619</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17440175</v>
+        <v>17446557</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2844011</v>
+        <v>2850406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-04 02:08:53
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 3, 2026</t>
+    <t>October 4, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18916133</v>
+        <v>18927875</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2885965</v>
+        <v>2896285</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1149057</v>
+        <v>1149133</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37372</v>
+        <v>37448</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204712</v>
+        <v>204759</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51244</v>
+        <v>51291</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>230479</v>
+        <v>230583</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>66984</v>
+        <v>67088</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187396</v>
+        <v>187438</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36591</v>
+        <v>36633</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196680</v>
+        <v>196692</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39304</v>
+        <v>39316</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451167</v>
+        <v>451259</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68419</v>
+        <v>68511</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>800458</v>
+        <v>800610</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>193090</v>
+        <v>193242</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96069</v>
+        <v>96070</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7270</v>
+        <v>7271</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>257632</v>
+        <v>257982</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>72022</v>
+        <v>72372</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4105463</v>
+        <v>4106657</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1134871</v>
+        <v>1136065</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8038316</v>
+        <v>8041413</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>898973</v>
+        <v>902070</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3845869</v>
+        <v>3848339</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>677592</v>
+        <v>680062</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1339666</v>
+        <v>1341324</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>47791</v>
+        <v>49449</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346238</v>
+        <v>347660</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1101391</v>
+        <v>1103131</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>98869</v>
+        <v>100609</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>139190</v>
+        <v>139351</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>27869</v>
+        <v>28030</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6918507</v>
+        <v>6923031</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1275619</v>
+        <v>1279780</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17446557</v>
+        <v>17456335</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2850406</v>
+        <v>2859136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-05 01:34:25
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 4, 2026</t>
+    <t>October 5, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18927875</v>
+        <v>18935453</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2896285</v>
+        <v>2903526</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1149133</v>
+        <v>1149502</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37448</v>
+        <v>37817</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204759</v>
+        <v>204812</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51291</v>
+        <v>51344</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>230583</v>
+        <v>230940</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>67088</v>
+        <v>67445</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187438</v>
+        <v>187594</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36633</v>
+        <v>36789</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196692</v>
+        <v>196710</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39316</v>
+        <v>39334</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451259</v>
+        <v>451290</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68511</v>
+        <v>68542</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>800610</v>
+        <v>801025</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>193242</v>
+        <v>193657</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96070</v>
+        <v>96073</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7271</v>
+        <v>7274</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>257982</v>
+        <v>258393</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>72372</v>
+        <v>72783</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4106657</v>
+        <v>4108465</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1136065</v>
+        <v>1137873</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8041413</v>
+        <v>8043849</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>902070</v>
+        <v>904506</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3848339</v>
+        <v>3849394</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>680062</v>
+        <v>681117</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1341324</v>
+        <v>1342037</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>49449</v>
+        <v>50162</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347660</v>
+        <v>347997</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1103131</v>
+        <v>1103859</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>100609</v>
+        <v>101337</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>139351</v>
+        <v>139852</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28030</v>
+        <v>28531</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6923031</v>
+        <v>6926157</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1279780</v>
+        <v>1282835</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17456335</v>
+        <v>17463306</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2859136</v>
+        <v>2865787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-06 01:28:08
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 5, 2026</t>
+    <t>October 6, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18935453</v>
+        <v>18943352</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2903526</v>
+        <v>2910977</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1149502</v>
+        <v>1149608</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37817</v>
+        <v>37923</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204812</v>
+        <v>205151</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51344</v>
+        <v>51683</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>230940</v>
+        <v>231260</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>67445</v>
+        <v>67765</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187594</v>
+        <v>187724</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>36789</v>
+        <v>36919</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196710</v>
+        <v>196752</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39334</v>
+        <v>39376</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451290</v>
+        <v>451431</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68542</v>
+        <v>68683</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>801025</v>
+        <v>801161</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>193657</v>
+        <v>193793</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96073</v>
+        <v>96074</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7274</v>
+        <v>7275</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>258393</v>
+        <v>258540</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>72783</v>
+        <v>72930</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4108465</v>
+        <v>4110786</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1137873</v>
+        <v>1140194</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8043849</v>
+        <v>8045948</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>904506</v>
+        <v>906605</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3849394</v>
+        <v>3850946</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>681117</v>
+        <v>682669</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1342037</v>
+        <v>1342848</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>50162</v>
+        <v>50973</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347997</v>
+        <v>348445</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1103859</v>
+        <v>1104507</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>101337</v>
+        <v>101985</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>139852</v>
+        <v>139872</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28531</v>
+        <v>28551</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6926157</v>
+        <v>6929699</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1282835</v>
+        <v>1286269</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17463306</v>
+        <v>17470520</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2865787</v>
+        <v>2872665</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-08 01:31:48
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 7, 2026</t>
+    <t>October 8, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18949610</v>
+        <v>18958365</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2917178</v>
+        <v>2925340</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1149645</v>
+        <v>1149891</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>37960</v>
+        <v>38206</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>205278</v>
+        <v>205419</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51810</v>
+        <v>51951</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231490</v>
+        <v>231502</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>67995</v>
+        <v>68007</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187863</v>
+        <v>187970</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37058</v>
+        <v>37165</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196833</v>
+        <v>196889</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39457</v>
+        <v>39513</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451486</v>
+        <v>451535</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68738</v>
+        <v>68787</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>801291</v>
+        <v>802390</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>193923</v>
+        <v>195022</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96091</v>
+        <v>96093</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7292</v>
+        <v>7294</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>258616</v>
+        <v>259062</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>73006</v>
+        <v>73452</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4113479</v>
+        <v>4116057</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1142887</v>
+        <v>1145465</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8047394</v>
+        <v>8049632</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>908051</v>
+        <v>910289</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3852061</v>
+        <v>3853791</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>683784</v>
+        <v>685514</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1343384</v>
+        <v>1344254</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>51509</v>
+        <v>52379</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348502</v>
+        <v>349095</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1104855</v>
+        <v>1105573</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>102333</v>
+        <v>103051</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>139935</v>
+        <v>139963</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28614</v>
+        <v>28642</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6932644</v>
+        <v>6936122</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1289231</v>
+        <v>1292669</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17476984</v>
+        <v>17485522</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2878962</v>
+        <v>2886942</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-09 01:33:52
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 8, 2026</t>
+    <t>October 9, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18958365</v>
+        <v>18964148</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2925340</v>
+        <v>2931163</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1149891</v>
+        <v>1150128</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>38206</v>
+        <v>38443</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>205419</v>
+        <v>205636</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>51951</v>
+        <v>52168</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231502</v>
+        <v>231568</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68007</v>
+        <v>68073</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>187970</v>
+        <v>188034</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37165</v>
+        <v>37229</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196889</v>
+        <v>196932</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39513</v>
+        <v>39556</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451535</v>
+        <v>451651</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68787</v>
+        <v>68903</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>802390</v>
+        <v>802610</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>195022</v>
+        <v>195242</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96093</v>
+        <v>96094</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7294</v>
+        <v>7295</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>259062</v>
+        <v>259492</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>73452</v>
+        <v>73882</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4116057</v>
+        <v>4119056</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1145465</v>
+        <v>1148464</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8049632</v>
+        <v>8050935</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>910289</v>
+        <v>911592</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3853791</v>
+        <v>3854492</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>685514</v>
+        <v>686215</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1344254</v>
+        <v>1344502</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>52379</v>
+        <v>52627</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349095</v>
+        <v>349055</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1105573</v>
+        <v>1105911</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>103051</v>
+        <v>103389</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>139963</v>
+        <v>140197</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28642</v>
+        <v>28876</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6936122</v>
+        <v>6939152</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1292669</v>
+        <v>1295849</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17485522</v>
+        <v>17491754</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2886942</v>
+        <v>2893072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-10 01:29:27
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 9, 2026</t>
+    <t>October 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18964148</v>
+        <v>18972388</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2931163</v>
+        <v>2938898</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1150128</v>
+        <v>1150232</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>38443</v>
+        <v>38547</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>205636</v>
+        <v>205786</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>52168</v>
+        <v>52318</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231568</v>
+        <v>231746</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68073</v>
+        <v>68251</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188034</v>
+        <v>188073</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37229</v>
+        <v>37268</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>196932</v>
+        <v>197082</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39556</v>
+        <v>39706</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>451651</v>
+        <v>452961</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>68903</v>
+        <v>70213</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>802610</v>
+        <v>802729</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>195242</v>
+        <v>195361</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96094</v>
+        <v>96208</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7295</v>
+        <v>7409</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>259492</v>
+        <v>259575</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>73882</v>
+        <v>73965</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4119056</v>
+        <v>4121394</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1148464</v>
+        <v>1150802</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8050935</v>
+        <v>8052916</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>911592</v>
+        <v>913573</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3854492</v>
+        <v>3856247</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>686215</v>
+        <v>687970</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1344502</v>
+        <v>1345513</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>52627</v>
+        <v>53638</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349055</v>
+        <v>349560</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1105911</v>
+        <v>1106535</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>103389</v>
+        <v>104013</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140197</v>
+        <v>140223</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28876</v>
+        <v>28902</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6939152</v>
+        <v>6942585</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1295849</v>
+        <v>1299075</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17491754</v>
+        <v>17499452</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2893072</v>
+        <v>2900336</v>
       </c>
     </row>
   </sheetData>
@@ -1177,7 +1177,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-12 01:41:14
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 11, 2026</t>
+    <t>October 12, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18976472</v>
+        <v>18979953</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2942969</v>
+        <v>2946469</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1150417</v>
+        <v>1150863</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>38732</v>
+        <v>39178</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>206018</v>
+        <v>206175</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>52550</v>
+        <v>52707</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231783</v>
+        <v>231834</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68288</v>
+        <v>68339</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188124</v>
+        <v>188144</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37319</v>
+        <v>37339</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197134</v>
+        <v>197154</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39758</v>
+        <v>39778</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>452996</v>
+        <v>453046</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70248</v>
+        <v>70298</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>803005</v>
+        <v>803845</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>195637</v>
+        <v>196477</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96225</v>
+        <v>96274</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7426</v>
+        <v>7475</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>259613</v>
+        <v>259798</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>74003</v>
+        <v>74188</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4122379</v>
+        <v>4123421</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1151787</v>
+        <v>1152829</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8054777</v>
+        <v>8056228</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>915434</v>
+        <v>916885</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3856976</v>
+        <v>3857357</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>688699</v>
+        <v>689080</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1345851</v>
+        <v>1346291</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>53976</v>
+        <v>54416</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349573</v>
+        <v>349554</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106665</v>
+        <v>1106803</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104143</v>
+        <v>104281</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140251</v>
+        <v>140299</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28930</v>
+        <v>28978</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6943961</v>
+        <v>6945344</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1300442</v>
+        <v>1301706</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17503270</v>
+        <v>17506570</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2904146</v>
+        <v>2907443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-13 01:35:54
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 12, 2026</t>
+    <t>October 13, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18979953</v>
+        <v>18985576</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2946469</v>
+        <v>2951941</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1150863</v>
+        <v>1150988</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39178</v>
+        <v>39303</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>206175</v>
+        <v>206511</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>52707</v>
+        <v>53043</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231834</v>
+        <v>231926</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68339</v>
+        <v>68431</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188144</v>
+        <v>188191</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37339</v>
+        <v>37386</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197154</v>
+        <v>197195</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39778</v>
+        <v>39819</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453046</v>
+        <v>453091</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70298</v>
+        <v>70343</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>803845</v>
+        <v>803987</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>196477</v>
+        <v>196619</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96274</v>
+        <v>96275</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7475</v>
+        <v>7476</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>259798</v>
+        <v>260283</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>74188</v>
+        <v>74673</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4123421</v>
+        <v>4125174</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1152829</v>
+        <v>1154582</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8056228</v>
+        <v>8058004</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>916885</v>
+        <v>918661</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3857357</v>
+        <v>3858529</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>689080</v>
+        <v>690252</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1346291</v>
+        <v>1346751</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>54416</v>
+        <v>54876</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349554</v>
+        <v>349705</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106803</v>
+        <v>1107075</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104281</v>
+        <v>104553</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140299</v>
+        <v>140338</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>28978</v>
+        <v>29017</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6945344</v>
+        <v>6947338</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1301706</v>
+        <v>1303731</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17506570</v>
+        <v>17512260</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2907443</v>
+        <v>2912946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-14 01:21:12
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 13, 2026</t>
+    <t>October 14, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18985576</v>
+        <v>18992790</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2951941</v>
+        <v>2958692</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1150988</v>
+        <v>1151151</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39303</v>
+        <v>39466</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>206511</v>
+        <v>206659</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>53043</v>
+        <v>53191</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>231926</v>
+        <v>232003</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68431</v>
+        <v>68508</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188191</v>
+        <v>188277</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37386</v>
+        <v>37472</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197195</v>
+        <v>197233</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39819</v>
+        <v>39857</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453091</v>
+        <v>453158</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70343</v>
+        <v>70410</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>803987</v>
+        <v>804101</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>196619</v>
+        <v>196733</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96275</v>
+        <v>96277</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7476</v>
+        <v>7478</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>260283</v>
+        <v>260862</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>74673</v>
+        <v>75252</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4125174</v>
+        <v>4126936</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1154582</v>
+        <v>1156344</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8058004</v>
+        <v>8059952</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>918661</v>
+        <v>920609</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3858529</v>
+        <v>3860121</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>690252</v>
+        <v>691844</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1346751</v>
+        <v>1347604</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>54876</v>
+        <v>55729</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349705</v>
+        <v>350168</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107075</v>
+        <v>1107650</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104553</v>
+        <v>105128</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140338</v>
+        <v>140359</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29017</v>
+        <v>29038</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6947338</v>
+        <v>6949813</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1303731</v>
+        <v>1306217</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17512260</v>
+        <v>17519350</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2912946</v>
+        <v>2919559</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-15 01:20:09
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 14, 2026</t>
+    <t>October 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18992790</v>
+        <v>19002314</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2958692</v>
+        <v>2967299</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151151</v>
+        <v>1151211</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39466</v>
+        <v>39526</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>206659</v>
+        <v>206912</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>53191</v>
+        <v>53444</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232003</v>
+        <v>232010</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68508</v>
+        <v>68515</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188277</v>
+        <v>188356</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37472</v>
+        <v>37551</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197233</v>
+        <v>197317</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39857</v>
+        <v>39941</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453158</v>
+        <v>453402</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70410</v>
+        <v>70654</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>804101</v>
+        <v>804213</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>196733</v>
+        <v>196845</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96277</v>
+        <v>96457</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7478</v>
+        <v>7658</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>260862</v>
+        <v>260911</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>75252</v>
+        <v>75301</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4126936</v>
+        <v>4129532</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1156344</v>
+        <v>1158940</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8059952</v>
+        <v>8061961</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>920609</v>
+        <v>922618</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3860121</v>
+        <v>3861866</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>691844</v>
+        <v>693589</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1347604</v>
+        <v>1348885</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>55729</v>
+        <v>57010</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>350168</v>
+        <v>351085</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107650</v>
+        <v>1108590</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>105128</v>
+        <v>106068</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140359</v>
+        <v>140395</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29038</v>
+        <v>29074</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6949813</v>
+        <v>6953520</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1306217</v>
+        <v>1309870</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17519350</v>
+        <v>17528692</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2919559</v>
+        <v>2927995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-16 01:18:09
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 15, 2026</t>
+    <t>October 16, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19002314</v>
+        <v>19008188</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2967299</v>
+        <v>2973536</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151211</v>
+        <v>1151298</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39526</v>
+        <v>39613</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>206912</v>
+        <v>207218</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>53444</v>
+        <v>53750</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232010</v>
+        <v>232161</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68515</v>
+        <v>68666</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188356</v>
+        <v>188400</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37551</v>
+        <v>37595</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197317</v>
+        <v>197356</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39941</v>
+        <v>39980</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453402</v>
+        <v>453532</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70654</v>
+        <v>70784</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>804213</v>
+        <v>805359</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>196845</v>
+        <v>197991</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>260911</v>
+        <v>261620</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>75301</v>
+        <v>76010</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4129532</v>
+        <v>4133723</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1158940</v>
+        <v>1163131</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8061961</v>
+        <v>8063351</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>922618</v>
+        <v>924008</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3861866</v>
+        <v>3862966</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>693589</v>
+        <v>694689</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348885</v>
+        <v>1348799</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57010</v>
+        <v>56924</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>351085</v>
+        <v>350722</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1108590</v>
+        <v>1108180</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>106068</v>
+        <v>105658</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140395</v>
+        <v>140447</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29074</v>
+        <v>29126</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6953520</v>
+        <v>6956162</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1309870</v>
+        <v>1312927</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17528692</v>
+        <v>17536120</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2927995</v>
+        <v>2935371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-17 01:19:55
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 16, 2026</t>
+    <t>October 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19008188</v>
+        <v>19011622</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2973536</v>
+        <v>2977532</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151298</v>
+        <v>1151489</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39613</v>
+        <v>39804</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>207218</v>
+        <v>207757</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>53750</v>
+        <v>54289</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232161</v>
+        <v>232372</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68666</v>
+        <v>68877</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188400</v>
+        <v>188464</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37595</v>
+        <v>37659</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197356</v>
+        <v>197455</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>39980</v>
+        <v>40079</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453532</v>
+        <v>453586</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70784</v>
+        <v>70838</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>805359</v>
+        <v>805515</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>197991</v>
+        <v>198147</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96457</v>
+        <v>96513</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7658</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>261620</v>
+        <v>261721</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>76010</v>
+        <v>76111</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4133723</v>
+        <v>4136504</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1163131</v>
+        <v>1165912</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8063351</v>
+        <v>8064824</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>924008</v>
+        <v>925481</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3862966</v>
+        <v>3863287</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>694689</v>
+        <v>695010</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348799</v>
+        <v>1348579</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56924</v>
+        <v>56704</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>350722</v>
+        <v>350160</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1108180</v>
+        <v>1107800</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>105658</v>
+        <v>105278</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140447</v>
+        <v>140468</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29126</v>
+        <v>29147</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6956162</v>
+        <v>6958262</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1312927</v>
+        <v>1315181</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17536120</v>
+        <v>17540052</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2935371</v>
+        <v>2939668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-18 01:23:43
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 17, 2026</t>
+    <t>October 18, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19011622</v>
+        <v>19013858</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2977532</v>
+        <v>2980304</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151489</v>
+        <v>1151727</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>39804</v>
+        <v>40042</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>207757</v>
+        <v>208044</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>54289</v>
+        <v>54576</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232372</v>
+        <v>232478</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68877</v>
+        <v>68983</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188464</v>
+        <v>188478</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37659</v>
+        <v>37673</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197455</v>
+        <v>197474</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40079</v>
+        <v>40098</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453586</v>
+        <v>453706</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70838</v>
+        <v>70958</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>805515</v>
+        <v>806823</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>198147</v>
+        <v>199455</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96513</v>
+        <v>96517</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7714</v>
+        <v>7718</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>261721</v>
+        <v>261825</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>76111</v>
+        <v>76215</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4136504</v>
+        <v>4137887</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1165912</v>
+        <v>1167295</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8064824</v>
+        <v>8066135</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>925481</v>
+        <v>926792</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3863287</v>
+        <v>3863516</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>695010</v>
+        <v>695239</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348579</v>
+        <v>1348310</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56704</v>
+        <v>56435</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>350160</v>
+        <v>349624</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107800</v>
+        <v>1107715</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>105278</v>
+        <v>105193</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140468</v>
+        <v>140671</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29147</v>
+        <v>29350</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6958262</v>
+        <v>6959027</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1315181</v>
+        <v>1316213</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17540052</v>
+        <v>17543091</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2939668</v>
+        <v>2942973</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-19 01:25:57
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 18, 2026</t>
+    <t>October 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19013858</v>
+        <v>19014098</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2980304</v>
+        <v>2981464</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151727</v>
+        <v>1151757</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40042</v>
+        <v>40072</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>208044</v>
+        <v>208194</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>54576</v>
+        <v>54726</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232478</v>
+        <v>232529</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>68983</v>
+        <v>69034</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188478</v>
+        <v>188597</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37673</v>
+        <v>37792</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197474</v>
+        <v>197539</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40098</v>
+        <v>40163</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>453706</v>
+        <v>454350</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>70958</v>
+        <v>71602</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>806823</v>
+        <v>806956</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>199455</v>
+        <v>199588</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>261825</v>
+        <v>262251</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>76215</v>
+        <v>76641</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4137887</v>
+        <v>4139556</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1167295</v>
+        <v>1168964</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8066135</v>
+        <v>8066936</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>926792</v>
+        <v>927593</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3863516</v>
+        <v>3863151</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>695239</v>
+        <v>694874</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348310</v>
+        <v>1347692</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56435</v>
+        <v>55817</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>349624</v>
+        <v>348704</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107715</v>
+        <v>1107196</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>105193</v>
+        <v>104674</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140671</v>
+        <v>140863</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29350</v>
+        <v>29542</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6959027</v>
+        <v>6959697</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1316213</v>
+        <v>1317087</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17543091</v>
+        <v>17544020</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2942973</v>
+        <v>2944613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-20 01:22:18
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 19, 2026</t>
+    <t>October 20, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19014098</v>
+        <v>19018735</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2981464</v>
+        <v>2986137</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151757</v>
+        <v>1151791</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40072</v>
+        <v>40106</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>208194</v>
+        <v>208552</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>54726</v>
+        <v>55084</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232529</v>
+        <v>232674</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69034</v>
+        <v>69179</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188597</v>
+        <v>188727</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37792</v>
+        <v>37922</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197539</v>
+        <v>197563</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40163</v>
+        <v>40187</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>454350</v>
+        <v>454600</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>71602</v>
+        <v>71852</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>806956</v>
+        <v>807355</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>199588</v>
+        <v>199987</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96517</v>
+        <v>96521</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7718</v>
+        <v>7722</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>262251</v>
+        <v>262821</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>76641</v>
+        <v>77211</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4139556</v>
+        <v>4141815</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1168964</v>
+        <v>1171223</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8066936</v>
+        <v>8068206</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>927593</v>
+        <v>928863</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3863151</v>
+        <v>3863864</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>694874</v>
+        <v>695587</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1347692</v>
+        <v>1347984</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>55817</v>
+        <v>56109</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348704</v>
+        <v>348668</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107196</v>
+        <v>1107324</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104674</v>
+        <v>104802</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140863</v>
+        <v>140874</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29542</v>
+        <v>29553</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6959697</v>
+        <v>6961932</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1317087</v>
+        <v>1319370</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17544020</v>
+        <v>17548903</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2944613</v>
+        <v>2949438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-21 01:23:34
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 20, 2026</t>
+    <t>October 21, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19018735</v>
+        <v>19020566</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2986137</v>
+        <v>2988376</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151791</v>
+        <v>1151834</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40106</v>
+        <v>40149</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>208552</v>
+        <v>208836</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55084</v>
+        <v>55368</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232674</v>
+        <v>232683</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69179</v>
+        <v>69188</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188727</v>
+        <v>188768</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37922</v>
+        <v>37963</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197563</v>
+        <v>197663</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40187</v>
+        <v>40287</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>454600</v>
+        <v>455324</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>71852</v>
+        <v>72576</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>807355</v>
+        <v>809113</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>199987</v>
+        <v>201745</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96521</v>
+        <v>96525</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7722</v>
+        <v>7726</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>262821</v>
+        <v>262925</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>77211</v>
+        <v>77315</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4141815</v>
+        <v>4143721</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1171223</v>
+        <v>1173129</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8068206</v>
+        <v>8068619</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>928863</v>
+        <v>929276</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3863864</v>
+        <v>3864252</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>695587</v>
+        <v>695975</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1347984</v>
+        <v>1347862</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56109</v>
+        <v>55987</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348668</v>
+        <v>348260</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107324</v>
+        <v>1106961</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104802</v>
+        <v>104439</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140874</v>
+        <v>140891</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29553</v>
+        <v>29570</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6961932</v>
+        <v>6963322</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1319370</v>
+        <v>1320837</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17548903</v>
+        <v>17550975</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2949438</v>
+        <v>2951830</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-22 01:20:40
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 21, 2026</t>
+    <t>October 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19020566</v>
+        <v>19025479</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2988376</v>
+        <v>2993251</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151834</v>
+        <v>1151866</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40149</v>
+        <v>40181</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>208836</v>
+        <v>208984</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55368</v>
+        <v>55516</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232683</v>
+        <v>232693</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69188</v>
+        <v>69198</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188768</v>
+        <v>188848</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>37963</v>
+        <v>38043</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197663</v>
+        <v>197696</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40287</v>
+        <v>40320</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>455324</v>
+        <v>455443</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>72576</v>
+        <v>72695</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>809113</v>
+        <v>809587</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>201745</v>
+        <v>202219</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96525</v>
+        <v>96644</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7726</v>
+        <v>7845</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>262925</v>
+        <v>263757</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>77315</v>
+        <v>78147</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4143721</v>
+        <v>4145673</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1173129</v>
+        <v>1175081</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8068619</v>
+        <v>8069737</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>929276</v>
+        <v>930394</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3864252</v>
+        <v>3865440</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>695975</v>
+        <v>697163</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1347862</v>
+        <v>1348443</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>55987</v>
+        <v>56568</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348260</v>
+        <v>348298</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106961</v>
+        <v>1106980</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104439</v>
+        <v>104458</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140891</v>
+        <v>140908</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29570</v>
+        <v>29587</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6963322</v>
+        <v>6965550</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1320837</v>
+        <v>1322936</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17550975</v>
+        <v>17555657</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2951830</v>
+        <v>2956448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-23 01:24:44
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 22, 2026</t>
+    <t>October 23, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19025479</v>
+        <v>19029083</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2993251</v>
+        <v>2997007</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151866</v>
+        <v>1151997</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40181</v>
+        <v>40312</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>208984</v>
+        <v>209088</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55516</v>
+        <v>55620</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232693</v>
+        <v>232818</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69198</v>
+        <v>69323</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188848</v>
+        <v>188910</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38043</v>
+        <v>38105</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197696</v>
+        <v>197751</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40320</v>
+        <v>40375</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>455443</v>
+        <v>455529</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>72695</v>
+        <v>72781</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>809587</v>
+        <v>809747</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>202219</v>
+        <v>202379</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>263757</v>
+        <v>264049</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>78147</v>
+        <v>78439</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4145673</v>
+        <v>4147468</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1175081</v>
+        <v>1176876</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8069737</v>
+        <v>8071043</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>930394</v>
+        <v>931700</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3865440</v>
+        <v>3865954</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>697163</v>
+        <v>697677</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348443</v>
+        <v>1348601</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56568</v>
+        <v>56726</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348298</v>
+        <v>348146</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106980</v>
+        <v>1106943</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104458</v>
+        <v>104421</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140908</v>
+        <v>140928</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29587</v>
+        <v>29607</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6965550</v>
+        <v>6967363</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1322936</v>
+        <v>1324773</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17555657</v>
+        <v>17559242</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2956448</v>
+        <v>2960149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-24 01:21:38
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 23, 2026</t>
+    <t>October 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19029083</v>
+        <v>19032411</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>2997007</v>
+        <v>3000668</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1151997</v>
+        <v>1152264</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40312</v>
+        <v>40579</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209088</v>
+        <v>209168</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55620</v>
+        <v>55700</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232818</v>
+        <v>232877</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69323</v>
+        <v>69382</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>188910</v>
+        <v>189031</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38105</v>
+        <v>38226</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197751</v>
+        <v>197828</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40375</v>
+        <v>40452</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>455529</v>
+        <v>455818</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>72781</v>
+        <v>73070</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>809747</v>
+        <v>810063</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>202379</v>
+        <v>202695</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96644</v>
+        <v>96645</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7845</v>
+        <v>7846</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264049</v>
+        <v>264512</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>78439</v>
+        <v>78902</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4147468</v>
+        <v>4149450</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1176876</v>
+        <v>1178858</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8071043</v>
+        <v>8071959</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>931700</v>
+        <v>932616</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3865954</v>
+        <v>3866442</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>697677</v>
+        <v>698165</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348601</v>
+        <v>1348615</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56726</v>
+        <v>56740</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>348146</v>
+        <v>347813</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106943</v>
+        <v>1107106</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104421</v>
+        <v>104584</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>140928</v>
+        <v>141026</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29607</v>
+        <v>29705</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6967363</v>
+        <v>6969450</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1324773</v>
+        <v>1326924</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17559242</v>
+        <v>17562738</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2960149</v>
+        <v>2963868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-25 01:22:41
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 24, 2026</t>
+    <t>October 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19032411</v>
+        <v>19035654</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3000668</v>
+        <v>3003990</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1152264</v>
+        <v>1152486</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40579</v>
+        <v>40801</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209168</v>
+        <v>209231</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55700</v>
+        <v>55763</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232877</v>
+        <v>232890</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69382</v>
+        <v>69395</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189031</v>
+        <v>189127</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38226</v>
+        <v>38322</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197828</v>
+        <v>197891</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40452</v>
+        <v>40515</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>455818</v>
+        <v>455970</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73070</v>
+        <v>73222</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>810063</v>
+        <v>810453</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>202695</v>
+        <v>203085</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264512</v>
+        <v>264558</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>78902</v>
+        <v>78948</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4149450</v>
+        <v>4150347</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1178858</v>
+        <v>1179755</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8071959</v>
+        <v>8073030</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>932616</v>
+        <v>933687</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3866442</v>
+        <v>3867166</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>698165</v>
+        <v>698889</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348615</v>
+        <v>1348921</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>56740</v>
+        <v>57046</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347813</v>
+        <v>347734</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107106</v>
+        <v>1107398</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104584</v>
+        <v>104876</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141026</v>
+        <v>141058</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29705</v>
+        <v>29737</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6969450</v>
+        <v>6970715</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1326924</v>
+        <v>1328200</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17562738</v>
+        <v>17565938</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2963868</v>
+        <v>2967114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-26 01:27:06
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 25, 2026</t>
+    <t>October 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19035654</v>
+        <v>19038290</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3003990</v>
+        <v>3006711</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1152486</v>
+        <v>1152545</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40801</v>
+        <v>40860</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209231</v>
+        <v>209303</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55763</v>
+        <v>55835</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232890</v>
+        <v>232899</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69395</v>
+        <v>69404</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189127</v>
+        <v>189188</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38322</v>
+        <v>38383</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197891</v>
+        <v>197925</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40515</v>
+        <v>40549</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>455970</v>
+        <v>456064</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73222</v>
+        <v>73316</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>810453</v>
+        <v>811078</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>203085</v>
+        <v>203710</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264558</v>
+        <v>264592</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>78948</v>
+        <v>78982</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4150347</v>
+        <v>4151339</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1179755</v>
+        <v>1180747</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8073030</v>
+        <v>8074046</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>933687</v>
+        <v>934703</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3867166</v>
+        <v>3867615</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>698889</v>
+        <v>699338</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1348921</v>
+        <v>1349155</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57046</v>
+        <v>57280</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347734</v>
+        <v>347649</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107398</v>
+        <v>1107400</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104876</v>
+        <v>104878</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141058</v>
+        <v>141086</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29737</v>
+        <v>29765</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6970715</v>
+        <v>6971865</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1328200</v>
+        <v>1329330</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17565938</v>
+        <v>17568417</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2967114</v>
+        <v>2969679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-27 01:25:36
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 26, 2026</t>
+    <t>October 27, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19038290</v>
+        <v>19042120</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3006711</v>
+        <v>3010820</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1152545</v>
+        <v>1152577</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40860</v>
+        <v>40892</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209303</v>
+        <v>209505</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>55835</v>
+        <v>56037</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>232899</v>
+        <v>233193</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69404</v>
+        <v>69698</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189188</v>
+        <v>189289</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38383</v>
+        <v>38484</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197925</v>
+        <v>197957</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40549</v>
+        <v>40581</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>456064</v>
+        <v>456183</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73316</v>
+        <v>73435</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>811078</v>
+        <v>811455</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>203710</v>
+        <v>204087</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96645</v>
+        <v>96647</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7846</v>
+        <v>7848</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264592</v>
+        <v>264647</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>78982</v>
+        <v>79037</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4151339</v>
+        <v>4153868</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1180747</v>
+        <v>1183276</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8074046</v>
+        <v>8075131</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>934703</v>
+        <v>935788</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3867615</v>
+        <v>3868083</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>699338</v>
+        <v>699806</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1349155</v>
+        <v>1349285</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57280</v>
+        <v>57410</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347649</v>
+        <v>347370</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107400</v>
+        <v>1107281</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104878</v>
+        <v>104759</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141086</v>
+        <v>141102</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29765</v>
+        <v>29781</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6971865</v>
+        <v>6974227</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1329330</v>
+        <v>1331700</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17568417</v>
+        <v>17572349</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2969679</v>
+        <v>2973836</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-28 01:09:41
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 27, 2026</t>
+    <t>October 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19042120</v>
+        <v>19045853</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3010820</v>
+        <v>3015141</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1152577</v>
+        <v>1152646</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40892</v>
+        <v>40961</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209505</v>
+        <v>209617</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>56037</v>
+        <v>56149</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>233193</v>
+        <v>233303</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69698</v>
+        <v>69808</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189289</v>
+        <v>189376</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38484</v>
+        <v>38571</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>197957</v>
+        <v>198143</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40581</v>
+        <v>40767</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>456183</v>
+        <v>456245</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73435</v>
+        <v>73497</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>811455</v>
+        <v>811758</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>204087</v>
+        <v>204390</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96647</v>
+        <v>96704</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7848</v>
+        <v>7905</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264647</v>
+        <v>264724</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>79037</v>
+        <v>79114</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4153868</v>
+        <v>4156929</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1183276</v>
+        <v>1186337</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8075131</v>
+        <v>8076052</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>935788</v>
+        <v>936709</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3868083</v>
+        <v>3868734</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>699806</v>
+        <v>700457</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1349285</v>
+        <v>1349139</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57410</v>
+        <v>57264</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347370</v>
+        <v>346782</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107281</v>
+        <v>1106999</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104759</v>
+        <v>104477</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141102</v>
+        <v>141218</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29781</v>
+        <v>29897</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6974227</v>
+        <v>6976674</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1331700</v>
+        <v>1334298</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17572349</v>
+        <v>17576655</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2973836</v>
+        <v>2978489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-29 01:09:30
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 28, 2026</t>
+    <t>October 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19045853</v>
+        <v>19052621</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3015141</v>
+        <v>3021664</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1152646</v>
+        <v>1153012</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>40961</v>
+        <v>41327</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209617</v>
+        <v>209746</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>56149</v>
+        <v>56278</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>233303</v>
+        <v>233319</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69808</v>
+        <v>69824</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189376</v>
+        <v>189418</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38571</v>
+        <v>38613</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>198143</v>
+        <v>198183</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40767</v>
+        <v>40807</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>456245</v>
+        <v>456427</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73497</v>
+        <v>73679</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>811758</v>
+        <v>811952</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>204390</v>
+        <v>204584</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264724</v>
+        <v>264821</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>79114</v>
+        <v>79211</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4156929</v>
+        <v>4159431</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1186337</v>
+        <v>1188839</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8076052</v>
+        <v>8077450</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>936709</v>
+        <v>938107</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3868734</v>
+        <v>3870311</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>700457</v>
+        <v>702034</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1349139</v>
+        <v>1349852</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57264</v>
+        <v>57977</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>346782</v>
+        <v>347027</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1106999</v>
+        <v>1107313</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104477</v>
+        <v>104791</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141218</v>
+        <v>141237</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29897</v>
+        <v>29916</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6976674</v>
+        <v>6979714</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1334298</v>
+        <v>1337231</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17576655</v>
+        <v>17583189</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2978489</v>
+        <v>2984788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-30 01:08:44
</commit_message>
<xml_diff>
--- a/assets/Downloads_Summary.xlsx
+++ b/assets/Downloads_Summary.xlsx
@@ -125,7 +125,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 29, 2026</t>
+    <t>October 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19052621</v>
+        <v>19061515</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -541,7 +541,7 @@
         <v>7171646</v>
       </c>
       <c r="H2">
-        <v>3021664</v>
+        <v>3030040</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -549,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1153012</v>
+        <v>1153060</v>
       </c>
       <c r="C3">
         <v>66223</v>
@@ -567,7 +567,7 @@
         <v>82035</v>
       </c>
       <c r="H3">
-        <v>41327</v>
+        <v>41375</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>209746</v>
+        <v>209849</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>87361</v>
       </c>
       <c r="H4">
-        <v>56278</v>
+        <v>56381</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>233319</v>
+        <v>233447</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>85205</v>
       </c>
       <c r="H5">
-        <v>69824</v>
+        <v>69952</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>189418</v>
+        <v>189459</v>
       </c>
       <c r="C6">
         <v>2843</v>
@@ -645,7 +645,7 @@
         <v>82723</v>
       </c>
       <c r="H6">
-        <v>38613</v>
+        <v>38654</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -653,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>198183</v>
+        <v>198211</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>72563</v>
       </c>
       <c r="H7">
-        <v>40807</v>
+        <v>40835</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>456427</v>
+        <v>456442</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -697,7 +697,7 @@
         <v>112970</v>
       </c>
       <c r="H8">
-        <v>73679</v>
+        <v>73694</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -705,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>811952</v>
+        <v>812052</v>
       </c>
       <c r="C9">
         <v>19239</v>
@@ -723,7 +723,7 @@
         <v>385784</v>
       </c>
       <c r="H9">
-        <v>204584</v>
+        <v>204684</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>96704</v>
+        <v>96705</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>15796</v>
       </c>
       <c r="H10">
-        <v>7905</v>
+        <v>7906</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>264821</v>
+        <v>265356</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>163185</v>
       </c>
       <c r="H11">
-        <v>79211</v>
+        <v>79746</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +895,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4159431</v>
+        <v>4162154</v>
       </c>
       <c r="C2">
         <v>125488</v>
@@ -913,7 +913,7 @@
         <v>1121180</v>
       </c>
       <c r="H2">
-        <v>1188839</v>
+        <v>1191562</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -921,7 +921,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>8077450</v>
+        <v>8078976</v>
       </c>
       <c r="C3">
         <v>139084</v>
@@ -939,7 +939,7 @@
         <v>3394391</v>
       </c>
       <c r="H3">
-        <v>938107</v>
+        <v>939633</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -947,7 +947,7 @@
         <v>24</v>
       </c>
       <c r="B4">
-        <v>3870311</v>
+        <v>3872643</v>
       </c>
       <c r="C4">
         <v>260697</v>
@@ -965,7 +965,7 @@
         <v>1591575</v>
       </c>
       <c r="H4">
-        <v>702034</v>
+        <v>704366</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>1349852</v>
+        <v>1350386</v>
       </c>
       <c r="C5">
         <v>102432</v>
@@ -991,7 +991,7 @@
         <v>396672</v>
       </c>
       <c r="H5">
-        <v>57977</v>
+        <v>58511</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -999,7 +999,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>347027</v>
+        <v>347545</v>
       </c>
       <c r="C6">
         <v>2304</v>
@@ -1025,7 +1025,7 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>1107313</v>
+        <v>1108556</v>
       </c>
       <c r="C7">
         <v>25615</v>
@@ -1043,7 +1043,7 @@
         <v>421508</v>
       </c>
       <c r="H7">
-        <v>104791</v>
+        <v>106034</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1051,7 +1051,7 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>141237</v>
+        <v>141255</v>
       </c>
       <c r="C8">
         <v>21217</v>
@@ -1069,7 +1069,7 @@
         <v>23673</v>
       </c>
       <c r="H8">
-        <v>29916</v>
+        <v>29934</v>
       </c>
     </row>
   </sheetData>
@@ -1119,7 +1119,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>6979714</v>
+        <v>6983704</v>
       </c>
       <c r="C2">
         <v>676837</v>
@@ -1137,7 +1137,7 @@
         <v>1826038</v>
       </c>
       <c r="H2">
-        <v>1337231</v>
+        <v>1341251</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1145,7 +1145,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>17583189</v>
+        <v>17592099</v>
       </c>
       <c r="C3">
         <v>151103</v>
@@ -1163,7 +1163,7 @@
         <v>6905316</v>
       </c>
       <c r="H3">
-        <v>2984788</v>
+        <v>2993140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>